<commit_message>
Latest push working version Excel dependable version
</commit_message>
<xml_diff>
--- a/Engagement Scoping Tool - FCC.xlsx
+++ b/Engagement Scoping Tool - FCC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NavashanmugamAsokan\Desktop\Projects\Engagement Scoping Tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg573064-my.sharepoint.com/personal/dhakshnamoorthi_tamilmani_donyati_com/Documents/mastero ai/admin-scoping-app/engagement-scoping-tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BF8E667-47FF-4B51-B168-B4B7C179523F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{7BF8E667-47FF-4B51-B168-B4B7C179523F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EC7FCD5-46C4-4B6C-AE5B-0D3BDC36E8B8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="832" xr2:uid="{AA176829-270E-447A-BC90-ED156939CE6E}"/>
+    <workbookView xWindow="10220" yWindow="0" windowWidth="10510" windowHeight="10993" tabRatio="832" xr2:uid="{AA176829-270E-447A-BC90-ED156939CE6E}"/>
   </bookViews>
   <sheets>
     <sheet name="Scope Definition" sheetId="4" r:id="rId1"/>
@@ -1937,13 +1937,8 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1" tint="0.499984740745262"/>
+        <color theme="0"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1962,8 +1957,13 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
+        <color theme="1" tint="0.499984740745262"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -2014,15 +2014,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>9</xdr:col>
-          <xdr:colOff>552450</xdr:colOff>
+          <xdr:colOff>552734</xdr:colOff>
           <xdr:row>5</xdr:row>
-          <xdr:rowOff>12700</xdr:rowOff>
+          <xdr:rowOff>13648</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>14</xdr:col>
-          <xdr:colOff>660400</xdr:colOff>
+          <xdr:colOff>661916</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>40943</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2054,7 +2054,7 @@
             </a:ln>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="45720" tIns="32004" rIns="45720" bIns="32004" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="27432" rIns="36576" bIns="27432" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="ctr" rtl="0">
@@ -2518,22 +2518,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D93A19B7-A902-4BD0-880D-85DEFBB71085}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="B3:Z124"/>
-  <sheetFormatPr defaultColWidth="9.23046875" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.25" defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.23046875" style="30"/>
-    <col min="2" max="2" width="45.765625" style="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.84375" style="31" customWidth="1"/>
-    <col min="4" max="4" width="22.84375" style="30" customWidth="1"/>
-    <col min="5" max="5" width="7.23046875" style="30" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="26.15234375" style="30" customWidth="1"/>
-    <col min="7" max="7" width="40.4609375" style="30" customWidth="1"/>
-    <col min="8" max="8" width="20.765625" style="30" customWidth="1"/>
-    <col min="9" max="10" width="9.23046875" style="30"/>
-    <col min="11" max="11" width="45.23046875" style="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.23046875" style="30"/>
+    <col min="1" max="1" width="9.25" style="30"/>
+    <col min="2" max="2" width="27.83203125" style="30" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" style="31" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" style="30" customWidth="1"/>
+    <col min="5" max="5" width="7.25" style="30" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" style="30" customWidth="1"/>
+    <col min="7" max="7" width="40.5" style="30" customWidth="1"/>
+    <col min="8" max="8" width="20.75" style="30" customWidth="1"/>
+    <col min="9" max="10" width="9.25" style="30"/>
+    <col min="11" max="11" width="45.25" style="30" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.25" style="30"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B3" s="42" t="s">
         <v>254</v>
       </c>
@@ -2550,7 +2550,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="4" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:26" x14ac:dyDescent="0.25">
       <c r="Y4" s="30" t="s">
         <v>91</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B5" s="32" t="s">
         <v>25</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
         <v>5</v>
       </c>
@@ -2601,7 +2601,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B7" s="27" t="s">
         <v>130</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
         <v>136</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B9" s="27" t="s">
         <v>267</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B10" s="27" t="s">
         <v>133</v>
       </c>
@@ -2691,7 +2691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B11" s="27" t="s">
         <v>6</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B12" s="27" t="s">
         <v>266</v>
       </c>
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B13" s="27" t="s">
         <v>131</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="14" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B14" s="27" t="s">
         <v>7</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B15" s="27" t="s">
         <v>19</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B16" s="27" t="s">
         <v>8</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="27" t="s">
         <v>132</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="27" t="s">
         <v>61</v>
       </c>
@@ -2892,7 +2892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="G19" s="30" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2908,7 +2908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="32" t="s">
         <v>26</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="27" t="s">
         <v>27</v>
       </c>
@@ -2954,7 +2954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="27" t="s">
         <v>214</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="27" t="s">
         <v>28</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="27" t="s">
         <v>134</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="27" t="s">
         <v>216</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="27" t="s">
         <v>29</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="27" t="s">
         <v>135</v>
       </c>
@@ -3096,7 +3096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="27" t="s">
         <v>155</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="27" t="s">
         <v>156</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="27" t="s">
         <v>265</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="27" t="s">
         <v>12</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="27" t="s">
         <v>30</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27" t="s">
         <v>31</v>
       </c>
@@ -3210,7 +3210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27" t="s">
         <v>32</v>
       </c>
@@ -3231,7 +3231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27" t="s">
         <v>124</v>
       </c>
@@ -3252,7 +3252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27" t="s">
         <v>33</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="27" t="s">
         <v>176</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G38" s="30" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3304,7 +3304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="32" t="s">
         <v>215</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27" t="s">
         <v>35</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27" t="s">
         <v>36</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G42" s="30" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3394,7 +3394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="32" t="s">
         <v>204</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" s="27" t="s">
         <v>268</v>
       </c>
@@ -3439,7 +3439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="27" t="s">
         <v>34</v>
       </c>
@@ -3471,7 +3471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="27" t="s">
         <v>217</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="27" t="s">
         <v>269</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G48" s="30" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3523,7 +3523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="32" t="s">
         <v>37</v>
       </c>
@@ -3540,7 +3540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="27" t="s">
         <v>222</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="27" t="s">
         <v>38</v>
       </c>
@@ -3604,7 +3604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G52" s="30" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3614,7 +3614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="32" t="s">
         <v>39</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="27" t="s">
         <v>221</v>
       </c>
@@ -3663,7 +3663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="27" t="s">
         <v>120</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" s="27" t="s">
         <v>121</v>
       </c>
@@ -3705,7 +3705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" s="27" t="s">
         <v>202</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C58" s="40"/>
       <c r="G58" s="30" t="str">
         <f t="shared" si="0"/>
@@ -3737,7 +3737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B59" s="32" t="s">
         <v>40</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B60" s="27" t="s">
         <v>41</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B61" s="27" t="s">
         <v>45</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B62" s="27" t="s">
         <v>42</v>
       </c>
@@ -3821,7 +3821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B63" s="27" t="s">
         <v>43</v>
       </c>
@@ -3844,7 +3844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B64" s="27" t="s">
         <v>44</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G65" s="30" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -3877,7 +3877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B66" s="32" t="s">
         <v>46</v>
       </c>
@@ -3891,7 +3891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B67" s="27" t="s">
         <v>47</v>
       </c>
@@ -3914,7 +3914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B68" s="27" t="s">
         <v>48</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B69" s="27" t="s">
         <v>49</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B70" s="27" t="s">
         <v>50</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B71" s="27" t="s">
         <v>51</v>
       </c>
@@ -4002,7 +4002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B72" s="27" t="s">
         <v>52</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B73" s="27" t="s">
         <v>141</v>
       </c>
@@ -4046,7 +4046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G74" s="30" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -4056,7 +4056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B75" s="32" t="s">
         <v>22</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B76" s="27" t="s">
         <v>59</v>
       </c>
@@ -4094,7 +4094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B77" s="27" t="s">
         <v>23</v>
       </c>
@@ -4115,7 +4115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B78" s="27" t="s">
         <v>60</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B79" s="27" t="s">
         <v>24</v>
       </c>
@@ -4157,7 +4157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B81" s="32" t="s">
         <v>53</v>
       </c>
@@ -4171,7 +4171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B82" s="27" t="s">
         <v>54</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B83" s="27" t="s">
         <v>55</v>
       </c>
@@ -4213,7 +4213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B84" s="27" t="s">
         <v>56</v>
       </c>
@@ -4234,7 +4234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B85" s="27" t="s">
         <v>57</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B86" s="27" t="s">
         <v>58</v>
       </c>
@@ -4278,7 +4278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B88" s="32" t="s">
         <v>257</v>
       </c>
@@ -4291,7 +4291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B89" s="27" t="s">
         <v>259</v>
       </c>
@@ -4312,7 +4312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B90" s="27" t="s">
         <v>260</v>
       </c>
@@ -4333,7 +4333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B92" s="32" t="s">
         <v>62</v>
       </c>
@@ -4346,7 +4346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B93" s="27" t="s">
         <v>63</v>
       </c>
@@ -4367,7 +4367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B94" s="27" t="s">
         <v>64</v>
       </c>
@@ -4388,7 +4388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B95" s="27" t="s">
         <v>66</v>
       </c>
@@ -4409,13 +4409,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G96" s="30" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="97" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B97" s="32" t="s">
         <v>137</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B98" s="27" t="s">
         <v>65</v>
       </c>
@@ -4449,7 +4449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B99" s="27" t="s">
         <v>220</v>
       </c>
@@ -4470,13 +4470,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G100" s="30" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="101" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B101" s="32" t="s">
         <v>154</v>
       </c>
@@ -4489,7 +4489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B102" s="27" t="s">
         <v>160</v>
       </c>
@@ -4509,72 +4509,72 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:8" x14ac:dyDescent="0.25">
       <c r="E103" s="30">
         <f>SUM(E6:E102)</f>
         <v>130</v>
       </c>
     </row>
-    <row r="105" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C105" s="40"/>
       <c r="H105" s="41"/>
     </row>
-    <row r="108" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:8" x14ac:dyDescent="0.25">
       <c r="H108" s="41"/>
     </row>
-    <row r="116" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C116" s="40"/>
     </row>
-    <row r="121" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C121" s="40"/>
     </row>
-    <row r="124" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C124" s="40"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A7:C8 J7:XFD8 E7:F8">
-    <cfRule type="expression" dxfId="9" priority="12">
+  <conditionalFormatting sqref="A7:F8">
+    <cfRule type="expression" dxfId="9" priority="6">
       <formula>$C$6&lt;&gt;"YES"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A13:C13 J13 E13:F13 L13:XFD13">
-    <cfRule type="expression" dxfId="8" priority="11">
+  <conditionalFormatting sqref="A13:F13">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>$C$11&lt;&gt;"YES"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A17:C17 J17:XFD17 E17:F17 K18">
-    <cfRule type="expression" dxfId="7" priority="10">
+  <conditionalFormatting sqref="A17:F17">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>$C$16&lt;&gt;"YES"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24:C25 I24:XFD25 E24:F25 K25:L26">
-    <cfRule type="expression" dxfId="6" priority="7">
-      <formula>$C$23&lt;&gt;"YES"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D8">
-    <cfRule type="expression" dxfId="5" priority="6">
-      <formula>$C$6&lt;&gt;"YES"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D13">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>$C$11&lt;&gt;"YES"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>$C$16&lt;&gt;"YES"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D24:D25">
-    <cfRule type="expression" dxfId="2" priority="3">
+  <conditionalFormatting sqref="A24:F25">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>$C$23&lt;&gt;"YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>$C$7="NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I24:XFD25 K25:L26">
+    <cfRule type="expression" dxfId="4" priority="7">
+      <formula>$C$23&lt;&gt;"YES"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J13 L13:XFD13">
+    <cfRule type="expression" dxfId="3" priority="11">
+      <formula>$C$11&lt;&gt;"YES"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:XFD8">
+    <cfRule type="expression" dxfId="2" priority="12">
+      <formula>$C$6&lt;&gt;"YES"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J17:XFD17 K18">
+    <cfRule type="expression" dxfId="1" priority="10">
+      <formula>$C$16&lt;&gt;"YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K19:L19">
@@ -4596,15 +4596,15 @@
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
                     <xdr:col>9</xdr:col>
-                    <xdr:colOff>552450</xdr:colOff>
+                    <xdr:colOff>552734</xdr:colOff>
                     <xdr:row>5</xdr:row>
-                    <xdr:rowOff>12700</xdr:rowOff>
+                    <xdr:rowOff>13648</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>14</xdr:col>
-                    <xdr:colOff>660400</xdr:colOff>
+                    <xdr:colOff>661916</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>38100</xdr:rowOff>
+                    <xdr:rowOff>40943</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4621,187 +4621,187 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B3C5F9-2960-4004-8DA8-F0112045F2AD}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="C2:C47"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="218.23046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="218.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:3" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:3" ht="19.899999999999999" x14ac:dyDescent="0.35">
       <c r="C2" s="8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="3:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:3" ht="14.55" x14ac:dyDescent="0.25">
       <c r="C4" s="9" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="9" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="11" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="15" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="20" spans="3:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="3:3" ht="15.6" x14ac:dyDescent="0.35">
       <c r="C20" s="7" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="21" spans="3:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="3:3" ht="15.6" x14ac:dyDescent="0.35">
       <c r="C21" s="7" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="22" spans="3:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="3:3" ht="15.6" x14ac:dyDescent="0.35">
       <c r="C22" s="7" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C25" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C31" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C32" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C38" s="1" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43" s="1" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C44" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C47" t="s">
         <v>219</v>
       </c>
@@ -4815,43 +4815,43 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FFC3484-AC13-4B4B-BDB8-D632F625B6E1}">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="C4:K24"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="255.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="8.765625" customWidth="1"/>
+    <col min="3" max="3" width="255.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="8.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:11" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:11" ht="14.55" x14ac:dyDescent="0.25">
       <c r="C4" s="9" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C6" s="14" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="9" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="10" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C14" s="25" t="s">
         <v>262</v>
       </c>
@@ -4880,7 +4880,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C15" s="17" t="s">
         <v>297</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C16" s="17" t="s">
         <v>293</v>
       </c>
@@ -4938,7 +4938,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C17" s="17" t="s">
         <v>299</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C18" s="17" t="s">
         <v>309</v>
       </c>
@@ -4996,7 +4996,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C19" s="17" t="s">
         <v>308</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C20" s="17" t="s">
         <v>300</v>
       </c>
@@ -5054,7 +5054,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C21" s="17" t="s">
         <v>301</v>
       </c>
@@ -5083,7 +5083,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="22" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C22" s="17" t="s">
         <v>302</v>
       </c>
@@ -5112,7 +5112,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C23" s="17" t="s">
         <v>303</v>
       </c>
@@ -5141,7 +5141,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C24" s="17" t="s">
         <v>304</v>
       </c>
@@ -5179,72 +5179,72 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D41DE2A-54C1-4E8B-A428-DD2CE26111FE}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="C4:C17"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="45.23046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:3" ht="14.55" x14ac:dyDescent="0.25">
       <c r="C4" s="9" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="6" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="7" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="11" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="12" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="14" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="15" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="16" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>242</v>
       </c>
@@ -5258,28 +5258,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BFB565C-5AE3-4537-9DC7-50CA3C2F2265}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="C1:AB24"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.4609375" customWidth="1"/>
-    <col min="2" max="2" width="1.23046875" customWidth="1"/>
-    <col min="3" max="3" width="1.4609375" customWidth="1"/>
-    <col min="4" max="4" width="26.61328125" customWidth="1"/>
-    <col min="5" max="5" width="10.765625" customWidth="1"/>
-    <col min="6" max="6" width="12.15234375" customWidth="1"/>
-    <col min="7" max="7" width="29.4609375" customWidth="1"/>
-    <col min="8" max="8" width="46.4609375" customWidth="1"/>
-    <col min="9" max="9" width="7.15234375" customWidth="1"/>
-    <col min="10" max="11" width="11.765625" customWidth="1"/>
-    <col min="15" max="15" width="9.23046875" customWidth="1"/>
-    <col min="16" max="16" width="11.15234375" customWidth="1"/>
-    <col min="17" max="18" width="13.61328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.765625" customWidth="1"/>
-    <col min="20" max="20" width="15.3828125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.15234375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.4609375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.5" customWidth="1"/>
+    <col min="2" max="2" width="1.25" customWidth="1"/>
+    <col min="3" max="3" width="1.5" customWidth="1"/>
+    <col min="4" max="4" width="26.58203125" customWidth="1"/>
+    <col min="5" max="5" width="10.75" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="7" max="7" width="29.5" customWidth="1"/>
+    <col min="8" max="8" width="46.5" customWidth="1"/>
+    <col min="9" max="9" width="7.1640625" customWidth="1"/>
+    <col min="10" max="11" width="11.75" customWidth="1"/>
+    <col min="15" max="15" width="9.25" customWidth="1"/>
+    <col min="16" max="16" width="11.1640625" customWidth="1"/>
+    <col min="17" max="18" width="13.58203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.75" customWidth="1"/>
+    <col min="20" max="20" width="15.4140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C1" s="6"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10"/>
@@ -5289,7 +5289,7 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
     </row>
-    <row r="3" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:28" x14ac:dyDescent="0.25">
       <c r="E3" s="5"/>
       <c r="J3" s="55" t="s">
         <v>261</v>
@@ -5307,7 +5307,7 @@
       <c r="U3" s="55"/>
       <c r="V3" s="55"/>
     </row>
-    <row r="4" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D4" s="16"/>
       <c r="E4" s="53" t="s">
         <v>140</v>
@@ -5356,7 +5356,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="5" spans="3:28" ht="41.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:28" ht="41.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D5" s="16"/>
       <c r="E5" s="54" t="s">
         <v>243</v>
@@ -5407,7 +5407,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D6" s="12" t="s">
         <v>71</v>
       </c>
@@ -5471,7 +5471,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D7" s="12" t="s">
         <v>75</v>
       </c>
@@ -5532,7 +5532,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D8" s="12" t="s">
         <v>72</v>
       </c>
@@ -5593,7 +5593,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="9" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D9" s="12" t="s">
         <v>73</v>
       </c>
@@ -5657,7 +5657,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:28" x14ac:dyDescent="0.25">
       <c r="D10" s="12" t="s">
         <v>74</v>
       </c>
@@ -5718,7 +5718,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="11" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:28" x14ac:dyDescent="0.25">
       <c r="H11" s="22" t="s">
         <v>203</v>
       </c>
@@ -5772,7 +5772,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="12" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:28" x14ac:dyDescent="0.25">
       <c r="H12" s="22" t="s">
         <v>215</v>
       </c>
@@ -5823,7 +5823,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:28" x14ac:dyDescent="0.25">
       <c r="H13" s="22" t="s">
         <v>204</v>
       </c>
@@ -5874,7 +5874,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="14" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:28" x14ac:dyDescent="0.25">
       <c r="H14" s="22" t="s">
         <v>37</v>
       </c>
@@ -5922,7 +5922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:28" x14ac:dyDescent="0.25">
       <c r="H15" s="22" t="s">
         <v>39</v>
       </c>
@@ -5970,7 +5970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="3:28" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:28" x14ac:dyDescent="0.25">
       <c r="H16" s="22" t="s">
         <v>40</v>
       </c>
@@ -6018,7 +6018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H17" s="22" t="s">
         <v>46</v>
       </c>
@@ -6066,7 +6066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H18" s="22" t="s">
         <v>22</v>
       </c>
@@ -6114,7 +6114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="19" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H19" s="23" t="s">
         <v>53</v>
       </c>
@@ -6162,7 +6162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H20" s="24" t="s">
         <v>257</v>
       </c>
@@ -6210,7 +6210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H21" s="24" t="s">
         <v>62</v>
       </c>
@@ -6258,7 +6258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H22" s="24" t="s">
         <v>137</v>
       </c>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="8:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="8:22" x14ac:dyDescent="0.25">
       <c r="I24">
         <f>SUM(I6:I22)</f>
         <v>1892.5</v>
@@ -6378,19 +6378,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8BA6D14-B405-4F02-827A-6DB3AFD9B3B8}">
   <sheetPr codeName="Sheet17"/>
   <dimension ref="A3:J132"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="52.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.84375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.15234375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="14.4609375" customWidth="1"/>
-    <col min="7" max="7" width="16.15234375" customWidth="1"/>
-    <col min="8" max="8" width="9.765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.765625" customWidth="1"/>
+    <col min="2" max="2" width="52.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.1640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.5" customWidth="1"/>
+    <col min="7" max="7" width="16.1640625" customWidth="1"/>
+    <col min="8" max="8" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.75" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>212</v>
@@ -6414,7 +6414,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>177</v>
       </c>
@@ -6435,7 +6435,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>178</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>179</v>
       </c>
@@ -6457,7 +6457,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>180</v>
       </c>
@@ -6468,7 +6468,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>181</v>
       </c>
@@ -6479,7 +6479,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>182</v>
       </c>
@@ -6490,7 +6490,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>183</v>
       </c>
@@ -6501,7 +6501,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>184</v>
       </c>
@@ -6512,10 +6512,10 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>185</v>
       </c>
@@ -6536,7 +6536,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>187</v>
       </c>
@@ -6547,7 +6547,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>186</v>
       </c>
@@ -6567,10 +6567,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>271</v>
       </c>
@@ -6591,7 +6591,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>188</v>
       </c>
@@ -6602,7 +6602,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>189</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>190</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>191</v>
       </c>
@@ -6635,7 +6635,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>192</v>
       </c>
@@ -6646,7 +6646,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>193</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>194</v>
       </c>
@@ -6668,7 +6668,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>195</v>
       </c>
@@ -6679,10 +6679,10 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>196</v>
       </c>
@@ -6703,7 +6703,7 @@
         <v>5.25</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>88</v>
       </c>
@@ -6714,7 +6714,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>225</v>
       </c>
@@ -6725,7 +6725,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>197</v>
       </c>
@@ -6736,7 +6736,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>198</v>
       </c>
@@ -6747,7 +6747,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>199</v>
       </c>
@@ -6758,10 +6758,10 @@
         <v>67</v>
       </c>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>200</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>201</v>
       </c>
@@ -6793,7 +6793,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>76</v>
       </c>
@@ -6805,7 +6805,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>93</v>
       </c>
@@ -6825,7 +6825,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>138</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>226</v>
       </c>
@@ -6857,7 +6857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>139</v>
       </c>
@@ -6877,7 +6877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>77</v>
       </c>
@@ -6888,7 +6888,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>78</v>
       </c>
@@ -6900,7 +6900,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>270</v>
       </c>
@@ -6912,7 +6912,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>94</v>
       </c>
@@ -6932,7 +6932,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>79</v>
       </c>
@@ -6943,7 +6943,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>80</v>
       </c>
@@ -6963,7 +6963,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>81</v>
       </c>
@@ -6975,7 +6975,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>95</v>
       </c>
@@ -6995,7 +6995,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>96</v>
       </c>
@@ -7015,7 +7015,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>97</v>
       </c>
@@ -7035,10 +7035,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C52" s="3"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="1" t="s">
         <v>203</v>
       </c>
@@ -7059,7 +7059,7 @@
         <v>12.0625</v>
       </c>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>98</v>
       </c>
@@ -7071,7 +7071,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>10</v>
       </c>
@@ -7083,7 +7083,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>99</v>
       </c>
@@ -7103,7 +7103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>9</v>
       </c>
@@ -7115,7 +7115,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>102</v>
       </c>
@@ -7127,7 +7127,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>100</v>
       </c>
@@ -7139,7 +7139,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>101</v>
       </c>
@@ -7151,7 +7151,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>206</v>
       </c>
@@ -7171,7 +7171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>103</v>
       </c>
@@ -7183,7 +7183,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>104</v>
       </c>
@@ -7195,7 +7195,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>105</v>
       </c>
@@ -7207,7 +7207,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
         <v>11</v>
       </c>
@@ -7219,7 +7219,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>213</v>
       </c>
@@ -7231,7 +7231,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>106</v>
       </c>
@@ -7243,7 +7243,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>168</v>
       </c>
@@ -7255,10 +7255,10 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C69" s="3"/>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B70" s="1" t="s">
         <v>215</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
       <c r="B71" t="s">
         <v>4</v>
@@ -7306,7 +7306,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
       <c r="B72" t="s">
         <v>108</v>
@@ -7330,10 +7330,10 @@
         <v>285</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C73" s="3"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B74" s="1" t="s">
         <v>204</v>
       </c>
@@ -7357,7 +7357,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
       <c r="B75" t="s">
         <v>286</v>
@@ -7381,7 +7381,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
       <c r="B76" t="s">
         <v>107</v>
@@ -7405,7 +7405,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" t="s">
         <v>205</v>
@@ -7418,7 +7418,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" t="s">
         <v>287</v>
@@ -7439,11 +7439,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
       <c r="C79" s="3"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B80" s="1" t="s">
         <v>37</v>
       </c>
@@ -7464,7 +7464,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" t="s">
         <v>224</v>
@@ -7485,7 +7485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" t="s">
         <v>109</v>
@@ -7506,10 +7506,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C83" s="3"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B84" s="1" t="s">
         <v>39</v>
       </c>
@@ -7530,7 +7530,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="B85" t="s">
         <v>21</v>
@@ -7554,7 +7554,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="B86" t="s">
         <v>122</v>
@@ -7575,7 +7575,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="B87" t="s">
         <v>123</v>
@@ -7596,7 +7596,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="B88" t="s">
         <v>207</v>
@@ -7617,10 +7617,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C89" s="3"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B90" s="1" t="s">
         <v>40</v>
       </c>
@@ -7641,7 +7641,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" t="s">
         <v>110</v>
@@ -7662,7 +7662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" t="s">
         <v>111</v>
@@ -7683,7 +7683,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" t="s">
         <v>112</v>
@@ -7704,7 +7704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" t="s">
         <v>113</v>
@@ -7725,7 +7725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="B95" t="s">
         <v>114</v>
@@ -7746,11 +7746,11 @@
         <v>32</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
       <c r="C96" s="3"/>
     </row>
-    <row r="97" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B97" s="1" t="s">
         <v>46</v>
       </c>
@@ -7771,7 +7771,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="98" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>119</v>
       </c>
@@ -7791,7 +7791,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="99" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>13</v>
       </c>
@@ -7811,7 +7811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>14</v>
       </c>
@@ -7831,7 +7831,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>15</v>
       </c>
@@ -7851,7 +7851,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>16</v>
       </c>
@@ -7871,7 +7871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>17</v>
       </c>
@@ -7891,7 +7891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>218</v>
       </c>
@@ -7911,13 +7911,13 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>219</v>
       </c>
       <c r="C105" s="3"/>
     </row>
-    <row r="106" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B106" s="1" t="s">
         <v>22</v>
       </c>
@@ -7938,7 +7938,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>115</v>
       </c>
@@ -7950,7 +7950,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="108" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>116</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="109" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>82</v>
       </c>
@@ -7974,7 +7974,7 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="110" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>117</v>
       </c>
@@ -7986,13 +7986,13 @@
         <v>NO</v>
       </c>
     </row>
-    <row r="111" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>219</v>
       </c>
       <c r="C111" s="3"/>
     </row>
-    <row r="112" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B112" s="1" t="s">
         <v>53</v>
       </c>
@@ -8013,7 +8013,7 @@
         <v>30.5</v>
       </c>
     </row>
-    <row r="113" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B113" t="s">
         <v>83</v>
       </c>
@@ -8025,7 +8025,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="114" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>84</v>
       </c>
@@ -8037,7 +8037,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="115" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
         <v>85</v>
       </c>
@@ -8049,7 +8049,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="116" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>118</v>
       </c>
@@ -8068,7 +8068,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="117" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
         <v>86</v>
       </c>
@@ -8080,10 +8080,10 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="118" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C118" s="3"/>
     </row>
-    <row r="119" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B119" s="1" t="s">
         <v>257</v>
       </c>
@@ -8104,7 +8104,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B120" t="s">
         <v>256</v>
       </c>
@@ -8116,7 +8116,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="121" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B121" t="s">
         <v>258</v>
       </c>
@@ -8128,13 +8128,13 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="122" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B122" t="s">
         <v>219</v>
       </c>
       <c r="C122" s="3"/>
     </row>
-    <row r="123" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B123" s="1" t="s">
         <v>62</v>
       </c>
@@ -8155,7 +8155,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="124" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B124" t="s">
         <v>87</v>
       </c>
@@ -8167,7 +8167,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="125" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B125" t="s">
         <v>88</v>
       </c>
@@ -8179,7 +8179,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="126" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B126" t="s">
         <v>18</v>
       </c>
@@ -8191,13 +8191,13 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="127" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
         <v>219</v>
       </c>
       <c r="C127" s="3"/>
     </row>
-    <row r="128" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B128" s="1" t="s">
         <v>137</v>
       </c>
@@ -8218,7 +8218,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="129" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
         <v>89</v>
       </c>
@@ -8230,7 +8230,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="130" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
         <v>90</v>
       </c>
@@ -8242,7 +8242,7 @@
         <v>YES</v>
       </c>
     </row>
-    <row r="131" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F131" t="s">
         <v>229</v>
       </c>
@@ -8253,7 +8253,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="132" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F132">
         <f>SUM(G5:G130)</f>
         <v>1892.5</v>
@@ -8276,13 +8276,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F144AA61-EA0A-4249-9EA6-54673F2A52CB}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="D7:M21"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="32.3828125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.4140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="4:13" ht="14" x14ac:dyDescent="0.3">
+    <row r="7" spans="4:13" ht="13.45" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="4:13" ht="14" x14ac:dyDescent="0.25">
       <c r="D8" s="44" t="s">
         <v>272</v>
       </c>
@@ -8314,7 +8314,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="4:13" ht="14.55" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D9" s="45" t="s">
         <v>273</v>
       </c>
@@ -8328,7 +8328,7 @@
       <c r="L9" s="57"/>
       <c r="M9" s="57"/>
     </row>
-    <row r="10" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D10" s="46" t="s">
         <v>274</v>
       </c>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="M10" s="47"/>
     </row>
-    <row r="11" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D11" s="46" t="s">
         <v>275</v>
       </c>
@@ -8388,7 +8388,7 @@
       </c>
       <c r="M11" s="47"/>
     </row>
-    <row r="12" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D12" s="46" t="s">
         <v>276</v>
       </c>
@@ -8418,7 +8418,7 @@
       </c>
       <c r="M12" s="47"/>
     </row>
-    <row r="13" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D13" s="46" t="s">
         <v>277</v>
       </c>
@@ -8442,7 +8442,7 @@
       <c r="L13" s="47"/>
       <c r="M13" s="47"/>
     </row>
-    <row r="14" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D14" s="46" t="s">
         <v>278</v>
       </c>
@@ -8472,7 +8472,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="15" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D15" s="46" t="s">
         <v>279</v>
       </c>
@@ -8502,7 +8502,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="16" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D16" s="46" t="s">
         <v>280</v>
       </c>
@@ -8530,7 +8530,7 @@
       </c>
       <c r="M16" s="47"/>
     </row>
-    <row r="17" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D17" s="46" t="s">
         <v>281</v>
       </c>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="M17" s="47"/>
     </row>
-    <row r="18" spans="4:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="4:13" ht="14" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D18" s="48" t="s">
         <v>282</v>
       </c>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="M18" s="47"/>
     </row>
-    <row r="21" spans="4:13" ht="14" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:13" ht="13.45" x14ac:dyDescent="0.25">
       <c r="K21" s="49">
         <v>7010</v>
       </c>
@@ -8613,313 +8613,313 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7DD1A3D-BA43-4A6A-817A-FCF02050F91F}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="B3:J189"/>
-  <sheetFormatPr defaultRowHeight="13.5" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.9" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="24.765625" customWidth="1"/>
-    <col min="3" max="12" width="8.765625" customWidth="1"/>
+    <col min="2" max="2" width="24.75" customWidth="1"/>
+    <col min="3" max="12" width="8.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" ht="14.55" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="4" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="8" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="9" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="11" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f>"Account dimension (~ "&amp;'Scope Definition'!D6&amp;"accounts) will be configured based on the current Chart of Accounts. " &amp; IF('Scope Definition'!C8="NO","No redesign of the Chart of Accounts is anticipated in the SOW.","CoA Rationalization will be performed.") &amp; " Standard Trial Balance will be incorporated into the Account dimension to support the following financial statements."</f>
         <v>Account dimension (~ 2000accounts) will be configured based on the current Chart of Accounts. CoA Rationalization will be performed. Standard Trial Balance will be incorporated into the Account dimension to support the following financial statements.</v>
       </c>
     </row>
-    <row r="16" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f>"Up to "&amp;'Scope Definition'!D7&amp;" Account alternate hierarchies will be developed"</f>
         <v>Up to 2 Account alternate hierarchies will be developed</v>
       </c>
     </row>
-    <row r="17" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f>"Entity - (~"&amp;'Scope Definition'!D11&amp;") will be configures based on the currenct structure. In addtion, up to "&amp;'Scope Definition'!D13&amp;" alternate hierarchies will be developed"</f>
         <v>Entity - (~25) will be configures based on the currenct structure. In addtion, up to 2 alternate hierarchies will be developed</v>
       </c>
     </row>
-    <row r="18" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <f>"Currency dimension will be configures with "&amp;'Scope Definition'!D9&amp; " Currencies.There will be "&amp;'Scope Definition'!D10&amp; " Reporting Currency"</f>
         <v>Currency dimension will be configures with 5 Currencies.There will be 2 Reporting Currency</v>
       </c>
     </row>
-    <row r="19" spans="2:2" ht="15.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:2" ht="15.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="B19" s="7" t="str">
         <f>IF('Scope Definition'!C31="YES", "Movement dimension will be configured to support Cash Flow and Roll-forward activities.", "Movement dimension will be configured to support Roll-forward activities.")</f>
         <v>Movement dimension will be configured to support Cash Flow and Roll-forward activities.</v>
       </c>
     </row>
-    <row r="20" spans="2:2" ht="15.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:2" ht="15.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="B20" s="7" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="2:2" ht="15.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:2" ht="15.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="B21" s="7" t="str">
         <f>"Custom dimensions will be leveraged to support additional reporting requirements. Specific use of "&amp;'Scope Definition'!D16&amp;" Custom Dimensions will be determined during requirements and design"</f>
         <v>Custom dimensions will be leveraged to support additional reporting requirements. Specific use of 2 Custom Dimensions will be determined during requirements and design</v>
       </c>
     </row>
-    <row r="22" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
         <f>IF('Scope Definition'!C17="NO", "Custom dimensions will have only one primary hierarchy", "Custom dimensions will have "&amp;'Scope Definition'!D17&amp; " alternate hierarchies")</f>
         <v>Custom dimensions will have 2 alternate hierarchies</v>
       </c>
     </row>
-    <row r="23" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B25" t="str">
         <f>IF('Scope Definition'!C21="YES","Standard elimination capabilities will be provided","Elimination is not in scope")</f>
         <v>Standard elimination capabilities will be provided</v>
       </c>
     </row>
-    <row r="26" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <f>IF('Scope Definition'!C23="YES","Consolidation Journal will be enabled","Journals are not in scope") &amp; " and " &amp; IF('Scope Definition'!C24="YES",'Scope Definition'!D24&amp; " Journal Template will be created", "Journal Templates are not in scope")</f>
         <v>Consolidation Journal will be enabled and 1 Journal Template will be created</v>
       </c>
     </row>
-    <row r="27" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
         <f>IF('Scope Definition'!C26="NO","Ownership Management is not in scope, " &amp; "No Equity pickup", "Ownership management will be enabled." )</f>
         <v>Ownership Management is not in scope, No Equity pickup</v>
       </c>
     </row>
-    <row r="28" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
         <f>IF('Scope Definition'!C29="YES","Partner Elimination will be enabled", " ")</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="29" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
         <f>IF('Scope Definition'!C30="YES","Configurable Consolidartion Rules will be used", " ")</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="30" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B30" t="str">
         <f>IF('Scope Definition'!C31="YES","Our of box Configuration of indirect Cash Flow will be used.", "Cash Flow is not in scope.")</f>
         <v>Our of box Configuration of indirect Cash Flow will be used.</v>
       </c>
     </row>
-    <row r="31" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B31" t="str">
         <f>IF('Scope Definition'!C32="YES","Supplemental Data Collection will be enabled.", " ")</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="32" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B32" t="str">
         <f>IF('Scope Definition'!C33="YES","Enterprise Journals will be enabled.", "")</f>
         <v/>
       </c>
     </row>
-    <row r="33" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B33" t="str">
         <f>IF('Scope Definition'!C34="YES","Approval Process will be used in the application.", "")</f>
         <v>Approval Process will be used in the application.</v>
       </c>
     </row>
-    <row r="34" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B34" t="str">
         <f>IF('Scope Definition'!C35="YES","Task Manager will be used in the application to support Financial Consolidation and Close.", "")</f>
         <v>Task Manager will be used in the application to support Financial Consolidation and Close.</v>
       </c>
     </row>
-    <row r="35" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B35" t="str">
         <f>IF('Scope Definition'!C36="YES","Audit will be enabled in the application as per requierement.", "")</f>
         <v/>
       </c>
     </row>
-    <row r="36" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="38" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
         <f>IF('Scope Definition'!C40="YES","Custom Data Forms – If required, up to " &amp; 'Scope Definition'!D40 &amp;" Custom Data Forms will be developed to support Financial Consolidation and Close.","")</f>
         <v>Custom Data Forms – If required, up to 5 Custom Data Forms will be developed to support Financial Consolidation and Close.</v>
       </c>
     </row>
-    <row r="39" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B40" t="str">
         <f>IF('Scope Definition'!C41="YES","Custom Dashboards – If required, up to " &amp; 'Scope Definition'!D41 &amp;" Custom Dashboards will be developed to support Financial Consolidation and Close.","")</f>
         <v/>
       </c>
     </row>
-    <row r="41" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="43" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B43" t="str">
         <f>IF('Scope Definition'!C44="YES","Custom Business Rules – If required, up to " &amp; 'Scope Definition'!D44 &amp;" Custom Business rules will be developed to support Financial Consolidation and Close.","")</f>
         <v>Custom Business Rules – If required, up to 3 Custom Business rules will be developed to support Financial Consolidation and Close.</v>
       </c>
     </row>
-    <row r="44" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B44" t="str">
         <f>IF('Scope Definition'!C45="YES","Member Formulas  – If required, up to " &amp; 'Scope Definition'!D45 &amp;" Member Formulas will be developed to support Financial Consolidation and Close.","")</f>
         <v>Member Formulas  – If required, up to 20 Member Formulas will be developed to support Financial Consolidation and Close.</v>
       </c>
     </row>
-    <row r="45" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B45" t="str">
         <f>IF('Scope Definition'!C46="YES","Translation override will be set up if required","")</f>
         <v>Translation override will be set up if required</v>
       </c>
     </row>
-    <row r="46" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B46" t="str">
         <f>IF('Scope Definition'!C47="YES","Calculate Movement rule will be enabled","")</f>
         <v/>
       </c>
     </row>
-    <row r="47" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="49" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="50" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="51" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="52" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="53" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="54" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="55" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="56" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="57" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="58" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="59" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="60" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="61" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="62" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="63" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="64" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="65" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="66" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="67" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="68" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="69" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="70" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="71" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="72" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="73" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="74" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="75" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="76" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="77" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="78" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="79" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="80" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="81" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="82" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="83" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="84" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="85" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="86" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="87" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="88" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="89" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="90" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="91" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="92" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="94" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="95" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="96" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="97" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="98" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="99" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="100" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="101" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="102" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="103" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="104" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="105" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="106" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="107" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="108" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="109" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="110" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="111" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="112" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="113" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="114" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="115" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="116" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="117" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="118" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="119" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="120" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="121" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="122" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="123" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="124" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="125" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="126" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="127" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="128" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="129" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="130" spans="2:4" collapsed="1" x14ac:dyDescent="0.3"/>
-    <row r="132" spans="2:4" ht="15" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="2:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="49" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="50" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="51" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="52" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="53" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="54" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="55" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="56" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="57" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="58" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="59" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="60" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="61" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="62" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="63" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="64" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="65" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="66" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="67" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="68" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="69" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="70" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="71" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="72" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="73" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="74" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="75" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="76" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="77" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="78" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="79" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="80" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="81" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="82" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="83" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="84" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="85" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="86" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="87" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="88" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="89" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="90" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="91" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="92" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="94" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="95" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="96" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="97" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="98" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="99" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="100" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="101" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="102" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="103" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="104" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="105" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="106" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="107" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="108" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="109" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="110" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="111" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="112" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="113" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="114" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="115" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="116" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="117" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="118" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="119" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="120" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="121" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="122" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="123" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="124" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="125" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="126" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="127" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="128" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="2:4" collapsed="1" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="2:4" ht="14.55" x14ac:dyDescent="0.25">
       <c r="B132" s="9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="133" spans="2:4" ht="15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:4" ht="14.55" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B133" s="9"/>
     </row>
-    <row r="134" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
         <v>162</v>
       </c>
@@ -8927,7 +8927,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="135" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
         <v>163</v>
       </c>
@@ -8935,7 +8935,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="136" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
         <v>164</v>
       </c>
@@ -8943,7 +8943,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="137" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
         <v>165</v>
       </c>
@@ -8951,7 +8951,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="138" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
         <v>9</v>
       </c>
@@ -8960,7 +8960,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B139" t="s">
         <v>103</v>
       </c>
@@ -8969,7 +8969,7 @@
         <v>Cash Flow</v>
       </c>
     </row>
-    <row r="140" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B140" t="s">
         <v>170</v>
       </c>
@@ -8978,7 +8978,7 @@
         <v>Journal Process</v>
       </c>
     </row>
-    <row r="141" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B141" t="s">
         <v>40</v>
       </c>
@@ -8987,7 +8987,7 @@
         <v>Integrations</v>
       </c>
     </row>
-    <row r="142" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B142" t="s">
         <v>166</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>Historical Data Source and Validations</v>
       </c>
     </row>
-    <row r="143" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B143" t="s">
         <v>22</v>
       </c>
@@ -9005,7 +9005,7 @@
         <v>Automations</v>
       </c>
     </row>
-    <row r="144" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>11</v>
       </c>
@@ -9014,7 +9014,7 @@
         <v>Approval Process</v>
       </c>
     </row>
-    <row r="145" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
         <v>106</v>
       </c>
@@ -9023,7 +9023,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B146" t="s">
         <v>104</v>
       </c>
@@ -9032,7 +9032,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B147" t="s">
         <v>105</v>
       </c>
@@ -9041,7 +9041,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B148" t="s">
         <v>167</v>
       </c>
@@ -9050,7 +9050,7 @@
         <v>Application Security</v>
       </c>
     </row>
-    <row r="149" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>168</v>
       </c>
@@ -9059,60 +9059,60 @@
         <v>Audit</v>
       </c>
     </row>
-    <row r="150" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="151" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="152" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="153" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="154" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="155" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="156" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="157" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="158" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="159" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="160" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="161" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="162" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="163" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="164" spans="2:10" collapsed="1" x14ac:dyDescent="0.3"/>
-    <row r="166" spans="2:10" ht="15" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="2:10" collapsed="1" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="2:10" ht="14.55" x14ac:dyDescent="0.25">
       <c r="B166" s="9" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="167" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="168" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B168" s="14" t="str">
         <f ca="1">"The engagement start date is " &amp; TEXT(TODAY(), "dd-mmm-yyyy")</f>
-        <v>The engagement start date is 18-Nov-2025</v>
-      </c>
-    </row>
-    <row r="169" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>The engagement start date is 05-Dec-2025</v>
+      </c>
+    </row>
+    <row r="169" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B169" t="str">
         <f ca="1">"The engagement end date is " &amp; TEXT(EOMONTH(TODAY(), ROUND(TotalDuration,0)),"dd-mmm-yyyy")</f>
-        <v>The engagement end date is 31-Jul-2026</v>
-      </c>
-    </row>
-    <row r="170" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>The engagement end date is 31-Aug-2026</v>
+      </c>
+    </row>
+    <row r="170" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B170" t="str">
         <f>"Go-live support will be provided and additional capabilities will be added per a subsequent Statement of Work expected to be started immediately following the completion of this Statement of Work."</f>
         <v>Go-live support will be provided and additional capabilities will be added per a subsequent Statement of Work expected to be started immediately following the completion of this Statement of Work.</v>
       </c>
     </row>
-    <row r="171" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B171" t="str">
         <f>"This SOW assumes " &amp; ROUND(TotalDuration,0) &amp; " months to complete Financial Consolidation and Close."</f>
         <v>This SOW assumes 8 months to complete Financial Consolidation and Close.</v>
       </c>
     </row>
-    <row r="172" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B172" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="173" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="174" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="175" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3"/>
-    <row r="176" spans="2:10" ht="27" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="2:10" ht="25.8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B176" s="20" t="s">
         <v>262</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B177" s="17" t="s">
         <v>297</v>
       </c>
@@ -9172,7 +9172,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="178" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B178" s="17" t="s">
         <v>293</v>
       </c>
@@ -9202,7 +9202,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="179" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B179" s="17" t="s">
         <v>299</v>
       </c>
@@ -9232,7 +9232,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="180" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B180" s="17" t="s">
         <v>309</v>
       </c>
@@ -9262,7 +9262,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="181" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B181" s="17" t="s">
         <v>308</v>
       </c>
@@ -9292,7 +9292,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="182" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B182" s="17" t="s">
         <v>300</v>
       </c>
@@ -9322,7 +9322,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="183" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B183" s="17" t="s">
         <v>301</v>
       </c>
@@ -9352,7 +9352,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="184" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B184" s="17" t="s">
         <v>310</v>
       </c>
@@ -9382,7 +9382,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="185" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B185" s="17" t="s">
         <v>302</v>
       </c>
@@ -9412,7 +9412,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="186" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B186" s="17" t="s">
         <v>303</v>
       </c>
@@ -9442,7 +9442,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="187" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B187" s="17" t="s">
         <v>304</v>
       </c>
@@ -9472,7 +9472,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="188" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B188" s="17" t="s">
         <v>305</v>
       </c>
@@ -9502,7 +9502,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="189" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B189" s="17" t="s">
         <v>306</v>
       </c>
@@ -9538,21 +9538,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006E5C2A45308F30418733145DE4F9BE17" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="17980c6fda1a973693bc55cfab4093ce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34a304f7-6f0b-43d9-9d9f-f2b435867f21" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae031883a5ce2be9cb3b9022b9de7ac4" ns2:_="">
     <xsd:import namespace="34a304f7-6f0b-43d9-9d9f-f2b435867f21"/>
@@ -9690,10 +9675,35 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6534E6B2-6821-49DF-A449-66880F1BB818}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{510610E9-2415-4A59-8182-0698721408CF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="34a304f7-6f0b-43d9-9d9f-f2b435867f21"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9715,19 +9725,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{510610E9-2415-4A59-8182-0698721408CF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6534E6B2-6821-49DF-A449-66880F1BB818}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="34a304f7-6f0b-43d9-9d9f-f2b435867f21"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>